<commit_message>
Update output path handling in prepare_region_context for solar and wind technologies
</commit_message>
<xml_diff>
--- a/1_msr_creator/control_file_msr_creator.xlsx
+++ b/1_msr_creator/control_file_msr_creator.xlsx
@@ -568,7 +568,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -632,9 +632,6 @@
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1005,7 +1002,7 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="46.5" customFormat="1" s="8">
       <c r="A2" s="7" t="s">
         <v>156</v>
       </c>
@@ -1016,7 +1013,7 @@
         <v>158</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5" customFormat="1" s="8">
       <c r="A3" s="7" t="s">
         <v>159</v>
       </c>
@@ -1264,7 +1261,7 @@
       <c r="B20" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="C20" s="22"/>
+      <c r="C20" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="5" t="s">
@@ -1273,7 +1270,7 @@
       <c r="B21" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C21" s="22"/>
+      <c r="C21" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="5" t="s">
@@ -1316,18 +1313,18 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5" customFormat="1" s="8">
       <c r="A2" s="7" t="s">
         <v>81</v>
       </c>
       <c r="B2" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5" customFormat="1" s="8">
       <c r="A3" s="7" t="s">
         <v>83</v>
       </c>
@@ -1338,18 +1335,18 @@
         <v>82</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5" customFormat="1" s="8">
       <c r="A4" s="7" t="s">
         <v>84</v>
       </c>
       <c r="B4" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5" customFormat="1" s="8">
       <c r="A5" s="7" t="s">
         <v>85</v>
       </c>
@@ -1360,7 +1357,7 @@
         <v>82</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5" customFormat="1" s="8">
       <c r="A6" s="7" t="s">
         <v>86</v>
       </c>
@@ -1371,7 +1368,7 @@
         <v>87</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5" customFormat="1" s="8">
       <c r="A7" s="7" t="s">
         <v>88</v>
       </c>
@@ -1380,7 +1377,7 @@
       </c>
       <c r="C7" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5" customFormat="1" s="8">
       <c r="A8" s="7" t="s">
         <v>89</v>
       </c>
@@ -1391,7 +1388,7 @@
         <v>90</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="33" customFormat="1" s="8">
       <c r="A9" s="7" t="s">
         <v>91</v>
       </c>
@@ -1402,7 +1399,7 @@
         <v>92</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5" customFormat="1" s="8">
       <c r="A10" s="7" t="s">
         <v>93</v>
       </c>
@@ -1413,7 +1410,7 @@
         <v>87</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5" customFormat="1" s="8">
       <c r="A11" s="7" t="s">
         <v>94</v>
       </c>
@@ -1424,7 +1421,7 @@
         <v>87</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5" customFormat="1" s="8">
       <c r="A12" s="7" t="s">
         <v>95</v>
       </c>
@@ -1435,7 +1432,7 @@
         <v>96</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75" customFormat="1" s="8">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5" customFormat="1" s="8">
       <c r="A13" s="7" t="s">
         <v>97</v>
       </c>

</xml_diff>

<commit_message>
clarifications in control files
</commit_message>
<xml_diff>
--- a/1_msr_creator/control_file_msr_creator.xlsx
+++ b/1_msr_creator/control_file_msr_creator.xlsx
@@ -1,18 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/MSR code repo/1_msr_creator/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_70E5932D92A10A4BF24D02E33FBB750DE0EB9D5D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C03553C9-A2E8-4A37-A6EE-E1C0C3BB004D}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="paths"/>
-    <sheet r:id="rId2" sheetId="2" name="datasets"/>
-    <sheet r:id="rId3" sheetId="3" name="configurations"/>
-    <sheet r:id="rId4" sheetId="4" name="parameters"/>
+    <sheet name="paths" sheetId="1" r:id="rId1"/>
+    <sheet name="datasets" sheetId="2" r:id="rId2"/>
+    <sheet name="configurations" sheetId="3" r:id="rId3"/>
+    <sheet name="parameters" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -265,9 +271,6 @@
     <t>run_code_for_solar_pv</t>
   </si>
   <si>
-    <t xml:space="preserve">Options=[0-No, 1-Yes]. </t>
-  </si>
-  <si>
     <t>run_code_for_solar_csp</t>
   </si>
   <si>
@@ -502,14 +505,16 @@
     <t>C:\Dev\model_supply_regions\Model-Supply-Regions-MSR-Toolset\outputs</t>
   </si>
   <si>
-    <t>Folder path where ouputs are located.</t>
+    <t>Folder path where outputs are located.</t>
+  </si>
+  <si>
+    <t>Options=[0-No, 1-Yes]. Only select one at a time.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -569,129 +574,132 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="22">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C43" displayName="Table3" name="Table3" id="1" totalsRowShown="0">
-  <autoFilter ref="A1:C43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table5" displayName="Table5" ref="A1:C3" totalsRowShown="0">
+  <autoFilter ref="A1:C3" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="3">
-    <tableColumn name="parameters" id="1"/>
-    <tableColumn name="value" id="2"/>
-    <tableColumn name="comments" id="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="parameter"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="value"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="comments"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C13" displayName="Table4" name="Table4" id="2" totalsRowShown="0">
-  <autoFilter ref="A1:C13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table1" displayName="Table1" ref="A1:C22" totalsRowShown="0">
+  <autoFilter ref="A1:C22" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="3">
-    <tableColumn name="parameter" id="1"/>
-    <tableColumn name="value" id="2"/>
-    <tableColumn name="comments" id="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="parameter"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="value"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="comments"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C22" displayName="Table1" name="Table1" id="3" totalsRowShown="0">
-  <autoFilter ref="A1:C22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table4" displayName="Table4" ref="A1:C13" totalsRowShown="0">
+  <autoFilter ref="A1:C13" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="3">
-    <tableColumn name="parameter" id="1"/>
-    <tableColumn name="value" id="2"/>
-    <tableColumn name="comments" id="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="parameter"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="value"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="comments"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C3" displayName="Table5" name="Table5" id="4" totalsRowShown="0">
-  <autoFilter ref="A1:C3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table3" displayName="Table3" ref="A1:C43" totalsRowShown="0">
+  <autoFilter ref="A1:C43" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="3">
-    <tableColumn name="parameter" id="1"/>
-    <tableColumn name="value" id="2"/>
-    <tableColumn name="comments" id="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="parameters"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="value"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="comments"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -700,10 +708,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -741,71 +749,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -833,7 +841,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -856,11 +864,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -869,13 +877,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -885,7 +893,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -894,7 +902,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -903,7 +911,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -911,10 +919,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -979,19 +987,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="19" width="19.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="19" width="69.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="19" width="38.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="19.1796875" style="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="69.81640625" style="19" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.7265625" style="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5" customFormat="1" s="8">
+    <row r="1" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>80</v>
       </c>
@@ -1002,26 +1010,26 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="46.5" customFormat="1" s="8">
+    <row r="2" spans="1:3" s="8" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="C2" s="7" t="s">
+    </row>
+    <row r="3" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="7" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5" customFormat="1" s="8">
-      <c r="A3" s="7" t="s">
+      <c r="B3" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="7" t="s">
         <v>160</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -1033,19 +1041,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="17" width="38.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="17" width="35.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="17" width="38.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="38.1796875" style="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.453125" style="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.1796875" style="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row r="1" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>80</v>
       </c>
@@ -1056,228 +1064,228 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="5" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="5" t="s">
+      <c r="B3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="5" t="s">
+    </row>
+    <row r="4" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="5" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="5" t="s">
+      <c r="B4" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C4" s="5" t="s">
+    </row>
+    <row r="5" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
-      <c r="A5" s="5" t="s">
+      <c r="B5" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="C5" s="5" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="5" t="s">
+      <c r="B6" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="C6" s="5" t="s">
+    </row>
+    <row r="7" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="5" t="s">
+      <c r="B7" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="C7" s="5" t="s">
+    </row>
+    <row r="8" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="5" t="s">
+      <c r="B8" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="C8" s="5" t="s">
+    </row>
+    <row r="9" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="5" t="s">
+      <c r="B9" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="C9" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="C9" s="5" t="s">
+    </row>
+    <row r="10" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
-      <c r="A10" s="5" t="s">
+      <c r="B10" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="C10" s="5" t="s">
+    </row>
+    <row r="11" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="5" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
-      <c r="A11" s="5" t="s">
+      <c r="B11" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="C11" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="C11" s="5" t="s">
+    </row>
+    <row r="12" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
-      <c r="A12" s="5" t="s">
+      <c r="B12" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="C12" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="C12" s="5" t="s">
+    </row>
+    <row r="13" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
-      <c r="A13" s="5" t="s">
+      <c r="B13" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="C13" s="5" t="s">
+    </row>
+    <row r="14" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="5" t="s">
+      <c r="B14" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
-      <c r="A15" s="5" t="s">
+      <c r="B15" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
-      <c r="A16" s="5" t="s">
+      <c r="B16" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
-      <c r="A17" s="5" t="s">
+      <c r="B17" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="C17" s="5" t="s">
+    </row>
+    <row r="18" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="5" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
-      <c r="A18" s="5" t="s">
+      <c r="B18" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="C18" s="5" t="s">
+    </row>
+    <row r="19" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
-      <c r="A19" s="5" t="s">
+      <c r="B19" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="C19" s="5" t="s">
+    </row>
+    <row r="20" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
-      <c r="A20" s="5" t="s">
+      <c r="B20" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" s="5"/>
+    </row>
+    <row r="21" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="C20" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
-      <c r="A21" s="5" t="s">
+      <c r="B21" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5"/>
+    </row>
+    <row r="22" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C21" s="5"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
-      <c r="A22" s="5" t="s">
+      <c r="B22" s="5" t="s">
         <v>154</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>155</v>
       </c>
       <c r="C22" s="5"/>
     </row>
@@ -1290,19 +1298,19 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="19" width="52.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="21" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="19" width="65.29071428571429" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="52.7265625" style="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.7265625" style="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="65.26953125" style="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5" customFormat="1" s="8">
+    <row r="1" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>80</v>
       </c>
@@ -1313,7 +1321,7 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5" customFormat="1" s="8">
+    <row r="2" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
         <v>81</v>
       </c>
@@ -1321,126 +1329,126 @@
         <v>1</v>
       </c>
       <c r="C2" s="7" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="7" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5" customFormat="1" s="8">
-      <c r="A3" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="B3" s="9">
         <v>0</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5" customFormat="1" s="8">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B4" s="9">
         <v>0</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5" customFormat="1" s="8">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B5" s="9">
         <v>0</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5" customFormat="1" s="8">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B6" s="9">
         <v>0</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="7" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5" customFormat="1" s="8">
-      <c r="A7" s="7" t="s">
-        <v>88</v>
       </c>
       <c r="B7" s="9">
         <v>1</v>
       </c>
       <c r="C7" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5" customFormat="1" s="8">
+    <row r="8" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B8" s="9">
         <v>1</v>
       </c>
       <c r="C8" s="7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" s="8" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="7" t="s">
         <v>90</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="33" customFormat="1" s="8">
-      <c r="A9" s="7" t="s">
-        <v>91</v>
       </c>
       <c r="B9" s="9">
         <v>0</v>
       </c>
       <c r="C9" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="7" t="s">
         <v>92</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5" customFormat="1" s="8">
-      <c r="A10" s="7" t="s">
-        <v>93</v>
       </c>
       <c r="B10" s="9">
         <v>1</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5" customFormat="1" s="8">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B11" s="9">
         <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5" customFormat="1" s="8">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B12" s="9">
         <v>0</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="7" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5" customFormat="1" s="8">
-      <c r="A13" s="7" t="s">
-        <v>97</v>
       </c>
       <c r="B13" s="9">
         <v>0</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1452,19 +1460,19 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="17" width="38.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="18" width="16.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="19" width="69.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="38.7265625" style="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.54296875" style="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="69.81640625" style="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row r="1" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1475,14 +1483,14 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="33.75">
+    <row r="3" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
@@ -1493,7 +1501,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="33.75">
+    <row r="4" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>6</v>
       </c>
@@ -1504,7 +1512,7 @@
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="33.75">
+    <row r="5" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
@@ -1515,7 +1523,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="33.75">
+    <row r="6" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
@@ -1526,7 +1534,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="33.75">
+    <row r="7" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -1537,7 +1545,7 @@
         <v>13</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+    <row r="8" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>14</v>
       </c>
@@ -1548,7 +1556,7 @@
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
+    <row r="9" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>16</v>
       </c>
@@ -1559,7 +1567,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="60.75" customFormat="1" s="8">
+    <row r="10" spans="1:3" s="8" customFormat="1" ht="60.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
         <v>19</v>
       </c>
@@ -1570,7 +1578,7 @@
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5" customFormat="1" s="8">
+    <row r="11" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
         <v>21</v>
       </c>
@@ -1581,7 +1589,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5" customFormat="1" s="8">
+    <row r="12" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
         <v>23</v>
       </c>
@@ -1592,7 +1600,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="33.75" customFormat="1" s="8">
+    <row r="13" spans="1:3" s="8" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
         <v>25</v>
       </c>
@@ -1603,19 +1611,19 @@
         <v>26</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5" customFormat="1" s="8">
+    <row r="14" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="7"/>
       <c r="B14" s="9"/>
       <c r="C14" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
+    <row r="15" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="11" t="s">
         <v>27</v>
       </c>
       <c r="B15" s="12"/>
       <c r="C15" s="13"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="33.75">
+    <row r="16" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>28</v>
       </c>
@@ -1626,7 +1634,7 @@
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="33.75">
+    <row r="17" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
         <v>30</v>
       </c>
@@ -1637,7 +1645,7 @@
         <v>31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
+    <row r="18" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
         <v>32</v>
       </c>
@@ -1648,7 +1656,7 @@
         <v>33</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="60.75">
+    <row r="19" spans="1:3" ht="60.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>34</v>
       </c>
@@ -1659,7 +1667,7 @@
         <v>35</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="47.25">
+    <row r="20" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
         <v>36</v>
       </c>
@@ -1670,7 +1678,7 @@
         <v>37</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="33.75">
+    <row r="21" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
         <v>38</v>
       </c>
@@ -1681,7 +1689,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
+    <row r="22" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
         <v>40</v>
       </c>
@@ -1692,19 +1700,19 @@
         <v>41</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+    <row r="23" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5"/>
       <c r="B23" s="6"/>
       <c r="C23" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
+    <row r="24" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="11" t="s">
         <v>42</v>
       </c>
       <c r="B24" s="14"/>
       <c r="C24" s="15"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="32.25">
+    <row r="25" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>43</v>
       </c>
@@ -1715,7 +1723,7 @@
         <v>44</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="33.75">
+    <row r="26" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
         <v>45</v>
       </c>
@@ -1726,7 +1734,7 @@
         <v>46</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5">
+    <row r="27" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
         <v>47</v>
       </c>
@@ -1737,7 +1745,7 @@
         <v>33</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+    <row r="28" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
         <v>48</v>
       </c>
@@ -1748,7 +1756,7 @@
         <v>49</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5">
+    <row r="29" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
         <v>50</v>
       </c>
@@ -1759,7 +1767,7 @@
         <v>51</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+    <row r="30" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
         <v>52</v>
       </c>
@@ -1770,7 +1778,7 @@
         <v>54</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5">
+    <row r="31" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
         <v>55</v>
       </c>
@@ -1781,19 +1789,19 @@
         <v>57</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
+    <row r="32" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5"/>
       <c r="B32" s="6"/>
       <c r="C32" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="19.5">
+    <row r="33" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="11" t="s">
         <v>58</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="15"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
+    <row r="34" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>59</v>
       </c>
@@ -1804,7 +1812,7 @@
         <v>60</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
+    <row r="35" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>61</v>
       </c>
@@ -1815,7 +1823,7 @@
         <v>62</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="19.5">
+    <row r="36" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>63</v>
       </c>
@@ -1826,7 +1834,7 @@
         <v>33</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="19.5">
+    <row r="37" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
         <v>64</v>
       </c>
@@ -1837,7 +1845,7 @@
         <v>65</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
+    <row r="38" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
         <v>66</v>
       </c>
@@ -1848,7 +1856,7 @@
         <v>67</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
+    <row r="39" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
         <v>68</v>
       </c>
@@ -1859,7 +1867,7 @@
         <v>69</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="19.5">
+    <row r="40" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
         <v>70</v>
       </c>
@@ -1870,7 +1878,7 @@
         <v>71</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
+    <row r="41" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
         <v>72</v>
       </c>
@@ -1881,7 +1889,7 @@
         <v>73</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
+    <row r="42" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
         <v>74</v>
       </c>
@@ -1892,7 +1900,7 @@
         <v>76</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="19.5">
+    <row r="43" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
         <v>77</v>
       </c>

</xml_diff>

<commit_message>
remove resource relaxation step from MSR creator (deemed unnecessary + avoid rasterio problems)
</commit_message>
<xml_diff>
--- a/1_msr_creator/control_file_msr_creator.xlsx
+++ b/1_msr_creator/control_file_msr_creator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/MSR code repo/1_msr_creator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_70E5932D92A10A4BF24D02E33FBB750DE0EB9D5D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C03553C9-A2E8-4A37-A6EE-E1C0C3BB004D}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_70E5932D92A10A4BF24D02E33FBB750DE0EB9D5D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D537FBC-6969-4C8A-AEDB-CE28C5C155E0}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="paths" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="156">
   <si>
     <t>parameters</t>
   </si>
@@ -61,18 +61,6 @@
     <t>Maximum allowed elevation; pixels above this value are excluded. Unit: m above sea level.</t>
   </si>
   <si>
-    <t>resource_relaxation_step</t>
-  </si>
-  <si>
-    <t>Step size used to lower the resource threshold during the resource sufficiency iteration.</t>
-  </si>
-  <si>
-    <t>region_area_threshold</t>
-  </si>
-  <si>
-    <t>Maximum allowed cumulative MSR area of the region's total area. Unit: %.</t>
-  </si>
-  <si>
     <t>land_cover_classes</t>
   </si>
   <si>
@@ -295,18 +283,6 @@
     <t>Options=[0-No, 1-Yes].</t>
   </si>
   <si>
-    <t>perform_stage_4_resource_sufficiency_check_and_relaxation</t>
-  </si>
-  <si>
-    <t>Options=[0-No, 1-Yes]. Enable to relax thresholds for resource lagging regions</t>
-  </si>
-  <si>
-    <t>perform_stage_5_polygonization</t>
-  </si>
-  <si>
-    <t>perform_stage_6_attribution</t>
-  </si>
-  <si>
     <t>grid_buffered_search</t>
   </si>
   <si>
@@ -509,6 +485,12 @@
   </si>
   <si>
     <t>Options=[0-No, 1-Yes]. Only select one at a time.</t>
+  </si>
+  <si>
+    <t>perform_stage_4_polygonization</t>
+  </si>
+  <si>
+    <t>perform_stage_5_attribution</t>
   </si>
 </sst>
 </file>
@@ -680,8 +662,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table4" displayName="Table4" ref="A1:C13" totalsRowShown="0">
-  <autoFilter ref="A1:C13" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table4" displayName="Table4" ref="A1:C12" totalsRowShown="0">
+  <autoFilter ref="A1:C12" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="parameter"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="value"/>
@@ -692,8 +674,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table3" displayName="Table3" ref="A1:C43" totalsRowShown="0">
-  <autoFilter ref="A1:C43" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table3" displayName="Table3" ref="A1:C41" totalsRowShown="0">
+  <autoFilter ref="A1:C41" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="parameters"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="value"/>
@@ -1001,7 +983,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -1012,24 +994,24 @@
     </row>
     <row r="2" spans="1:3" s="8" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -1055,7 +1037,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1066,226 +1048,226 @@
     </row>
     <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="C20" s="5"/>
     </row>
     <row r="21" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="C21" s="5"/>
     </row>
     <row r="22" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="C22" s="5"/>
     </row>
@@ -1312,7 +1294,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B1" s="20" t="s">
         <v>1</v>
@@ -1323,62 +1305,62 @@
     </row>
     <row r="2" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B2" s="9">
         <v>1</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B3" s="9">
         <v>0</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B4" s="9">
         <v>0</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B5" s="9">
         <v>0</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B6" s="9">
         <v>0</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B7" s="9">
         <v>1</v>
@@ -1387,69 +1369,63 @@
     </row>
     <row r="8" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B8" s="9">
         <v>1</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="8" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
-        <v>90</v>
+        <v>154</v>
       </c>
       <c r="B9" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
-        <v>92</v>
+        <v>155</v>
       </c>
       <c r="B10" s="9">
         <v>1</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="B11" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B12" s="9">
         <v>0</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B13" s="9">
-        <v>0</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>97</v>
-      </c>
+      <c r="A13" s="19"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1538,30 +1514,30 @@
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="6">
-        <v>0.01</v>
+      <c r="B7" s="6" t="s">
+        <v>13</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="6">
+      <c r="A8" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="9">
         <v>5</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>17</v>
+      </c>
+      <c r="B9" s="10">
+        <v>8760</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>18</v>
@@ -1571,8 +1547,8 @@
       <c r="A10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="9">
-        <v>5</v>
+      <c r="B10" s="10">
+        <v>365</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>20</v>
@@ -1582,53 +1558,53 @@
       <c r="A11" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="10">
-        <v>8760</v>
+      <c r="B11" s="9">
+        <v>5</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="7"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="7"/>
+    </row>
+    <row r="13" spans="1:3" s="8" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="10">
-        <v>365</v>
-      </c>
-      <c r="C12" s="7" t="s">
+      <c r="B13" s="12"/>
+      <c r="C13" s="13"/>
+    </row>
+    <row r="14" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" s="8" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="7" t="s">
+      <c r="B14" s="6">
+        <v>4</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="9">
-        <v>5</v>
-      </c>
-      <c r="C13" s="7" t="s">
+    </row>
+    <row r="15" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" s="8" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="7"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="7"/>
-    </row>
-    <row r="15" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="11" t="s">
+      <c r="B15" s="6">
+        <v>3</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="12"/>
-      <c r="C15" s="13"/>
     </row>
     <row r="16" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B16" s="6">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>29</v>
@@ -1639,7 +1615,7 @@
         <v>30</v>
       </c>
       <c r="B17" s="6">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>31</v>
@@ -1661,7 +1637,7 @@
         <v>34</v>
       </c>
       <c r="B19" s="6">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>35</v>
@@ -1672,166 +1648,166 @@
         <v>36</v>
       </c>
       <c r="B20" s="6">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="5"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="7"/>
+    </row>
+    <row r="22" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B21" s="6">
-        <v>10</v>
-      </c>
-      <c r="C21" s="7" t="s">
+      <c r="B22" s="14"/>
+      <c r="C22" s="15"/>
+    </row>
+    <row r="23" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="5" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="s">
+      <c r="B23" s="6">
+        <v>4</v>
+      </c>
+      <c r="C23" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="6">
-        <v>33</v>
-      </c>
-      <c r="C22" s="7" t="s">
+    </row>
+    <row r="24" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="5"/>
-      <c r="B23" s="6"/>
-      <c r="C23" s="7"/>
-    </row>
-    <row r="24" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="11" t="s">
+      <c r="B24" s="6">
+        <v>3</v>
+      </c>
+      <c r="C24" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="14"/>
-      <c r="C24" s="15"/>
     </row>
     <row r="25" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>43</v>
       </c>
       <c r="B25" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="6">
+        <v>10</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>45</v>
-      </c>
-      <c r="B26" s="6">
-        <v>3</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" s="6">
+        <v>17</v>
+      </c>
+      <c r="C27" s="7" t="s">
         <v>47</v>
-      </c>
-      <c r="B27" s="6">
-        <v>5</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B28" s="6">
-        <v>10</v>
+      <c r="B28" s="6" t="s">
+        <v>49</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="B29" s="6">
-        <v>17</v>
+        <v>51</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>52</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C30" s="7" t="s">
+      <c r="A30" s="5"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="7"/>
+    </row>
+    <row r="31" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="11" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="5" t="s">
+      <c r="B31" s="16"/>
+      <c r="C31" s="15"/>
+    </row>
+    <row r="32" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B32" s="6">
+        <v>6</v>
+      </c>
+      <c r="C32" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C31" s="7" t="s">
+    </row>
+    <row r="33" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="5" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="5"/>
-      <c r="B32" s="6"/>
-      <c r="C32" s="7"/>
-    </row>
-    <row r="33" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="11" t="s">
+      <c r="B33" s="6">
+        <v>4</v>
+      </c>
+      <c r="C33" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="16"/>
-      <c r="C33" s="15"/>
     </row>
     <row r="34" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>59</v>
       </c>
       <c r="B34" s="6">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B35" s="6">
+        <v>5</v>
+      </c>
+      <c r="C35" s="7" t="s">
         <v>61</v>
-      </c>
-      <c r="B35" s="6">
-        <v>4</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B36" s="6">
+        <v>3</v>
+      </c>
+      <c r="C36" s="7" t="s">
         <v>63</v>
-      </c>
-      <c r="B36" s="6">
-        <v>20</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1839,7 +1815,7 @@
         <v>64</v>
       </c>
       <c r="B37" s="6">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="C37" s="7" t="s">
         <v>65</v>
@@ -1850,7 +1826,7 @@
         <v>66</v>
       </c>
       <c r="B38" s="6">
-        <v>3</v>
+        <v>1.96</v>
       </c>
       <c r="C38" s="7" t="s">
         <v>67</v>
@@ -1861,7 +1837,7 @@
         <v>68</v>
       </c>
       <c r="B39" s="6">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="C39" s="7" t="s">
         <v>69</v>
@@ -1871,46 +1847,26 @@
       <c r="A40" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B40" s="6">
-        <v>1.96</v>
+      <c r="B40" s="6" t="s">
+        <v>71</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B41" s="6">
-        <v>25</v>
+        <v>73</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>74</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B42" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C42" s="7" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>79</v>
-      </c>
-    </row>
+    </row>
+    <row r="42" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="43" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
further simpliciations of script 1 control file
</commit_message>
<xml_diff>
--- a/1_msr_creator/control_file_msr_creator.xlsx
+++ b/1_msr_creator/control_file_msr_creator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/26001 MSR tutorial/1_msr_creator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="177" documentId="13_ncr:1_{66067BA5-85F1-4566-9789-B17D8F553E15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{028A1EFA-09FA-4A90-89DE-F678E9173A35}"/>
+  <xr:revisionPtr revIDLastSave="180" documentId="13_ncr:1_{66067BA5-85F1-4566-9789-B17D8F553E15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88E9B0C5-8EE9-4459-9953-E7C1737280E5}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="paths" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="129">
   <si>
     <t>parameters</t>
   </si>
@@ -94,12 +94,6 @@
     <t>Maximum allowed terrain slope; pixels above this value are excluded. Unit: %</t>
   </si>
   <si>
-    <t>pv_spacing_factor</t>
-  </si>
-  <si>
-    <t>Solar PV spacing factor during the resource sufficiency check. Unit: %. Based on: https://www.irena.org/publications/2014/Aug/Estimating-the-Renewable-Energy-Potential-in-Africa-A-GIS-based-approach</t>
-  </si>
-  <si>
     <t>pv_land_discount_factor</t>
   </si>
   <si>
@@ -136,18 +130,6 @@
     <t>Installed CSP capacity per square kilometre of developed land. Unit: MW/km².</t>
   </si>
   <si>
-    <t>csp_land_classes</t>
-  </si>
-  <si>
-    <t>DNI bin edges used to group suitable csp areas during the resource sufficiency yield estimate. Unit: kWh/m²/day. Based on: https://www.irena.org/publications/2015/Oct/Renewable-Energy-Zones-for-the-Africa-Clean-Energy-Corridor.</t>
-  </si>
-  <si>
-    <t>csp_production_percentage_per_land_class</t>
-  </si>
-  <si>
-    <t>Annual production per DNI bin. Unit: %</t>
-  </si>
-  <si>
     <t>Wind parameters</t>
   </si>
   <si>
@@ -190,18 +172,6 @@
     <t>Share of technically suitable land assumed to be available for wind deployment. Unit: %.</t>
   </si>
   <si>
-    <t>wind_land_classes</t>
-  </si>
-  <si>
-    <t>Wind speed bin edges used to group suitable wind areas during the resource sufficiency yield estimate. Unit: m/s. Based on: https://www.irena.org/publications/2014/Aug/Estimating-the-Renewable-Energy-Potential-in-Africa-A-GIS-based-approach</t>
-  </si>
-  <si>
-    <t>wind_production_percentage_per_land_class</t>
-  </si>
-  <si>
-    <t>Annual production per wind speed bin. Unit: %</t>
-  </si>
-  <si>
     <t>parameter</t>
   </si>
   <si>
@@ -413,18 +383,6 @@
   </si>
   <si>
     <t>11, 14, 20, 30, 110, 120, 130, 140, 150, 180, 190, 200</t>
-  </si>
-  <si>
-    <t>0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18</t>
-  </si>
-  <si>
-    <t>0,7.84,21.40,31.01,38.47,44.57,49.72,54.19,58.12,61.65,64.83,67.74,70.42,72.90,75.20,77.36,79.39,81.30</t>
-  </si>
-  <si>
-    <t>0,0.5,1,1.5,2,2.5,3,3.5,4,4.5,5,5.5,6,6.5,7,7.5,8,8.5,9,9.5,10,10.5,11,11.5,12</t>
-  </si>
-  <si>
-    <t>0,0,0,0,0,1,3,6,9,13,18,24,30,37,43,48,54,58,61,64,65,66,66,65</t>
   </si>
   <si>
     <t>ECU_GRIP</t>
@@ -674,8 +632,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table3" displayName="Table3" ref="A1:C35" totalsRowShown="0">
-  <autoFilter ref="A1:C35" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table3" displayName="Table3" ref="A1:C30" totalsRowShown="0">
+  <autoFilter ref="A1:C30" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="parameters"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="value"/>
@@ -983,7 +941,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -994,24 +952,24 @@
     </row>
     <row r="2" spans="1:3" s="7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1037,7 +995,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1048,222 +1006,222 @@
     </row>
     <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B16"/>
       <c r="C16" s="5" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B20"/>
       <c r="C20" s="5"/>
     </row>
     <row r="21" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="C21" s="5"/>
     </row>
     <row r="22" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="C22" s="5"/>
     </row>
@@ -1290,7 +1248,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B1" s="15" t="s">
         <v>1</v>
@@ -1301,123 +1259,123 @@
     </row>
     <row r="2" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B2" s="18">
         <v>0</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B3" s="18">
         <v>0</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="B4" s="18">
         <v>1</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B5" s="18">
         <v>0</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="B6" s="8">
         <v>1</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B7" s="8">
         <v>1</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B8" s="8">
         <v>1</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="B9" s="8">
         <v>1</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="B10" s="8">
         <v>1</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="B11" s="8">
         <v>0</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B12" s="8">
         <v>0</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1513,7 +1471,7 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>13</v>
@@ -1575,149 +1533,149 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:3" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" s="7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B14">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:3" s="7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B15">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="5"/>
+      <c r="B16"/>
+      <c r="C16" s="6"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B16">
-        <v>33</v>
-      </c>
-      <c r="C16" s="6" t="s">
+      <c r="B17"/>
+      <c r="C17" s="11"/>
+    </row>
+    <row r="18" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="5" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="5"/>
-      <c r="B17"/>
-      <c r="C17" s="6"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" s="9" t="s">
+      <c r="B18">
+        <v>4</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B18"/>
-      <c r="C18" s="11"/>
-    </row>
-    <row r="19" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" s="5" t="s">
+      <c r="B20">
+        <v>10</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B20">
-        <v>5</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
         <v>33</v>
       </c>
       <c r="B21">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="5"/>
+      <c r="B22"/>
+      <c r="C22" s="6"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B22">
-        <v>17</v>
-      </c>
-      <c r="C22" s="6" t="s">
+      <c r="B23"/>
+      <c r="C23" s="11"/>
+    </row>
+    <row r="24" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" ht="58" x14ac:dyDescent="0.35">
-      <c r="A23" s="5" t="s">
+      <c r="B24">
+        <v>6</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B23" t="s">
-        <v>130</v>
-      </c>
-      <c r="C23" s="6" t="s">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" s="5" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" s="5" t="s">
+      <c r="B25">
+        <v>20</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B24" t="s">
-        <v>131</v>
-      </c>
-      <c r="C24" s="6" t="s">
+      <c r="B26">
+        <v>5</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A25" s="5"/>
-      <c r="B25"/>
-      <c r="C25" s="6"/>
-    </row>
-    <row r="26" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26"/>
-      <c r="C26" s="11"/>
     </row>
     <row r="27" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27">
+        <v>3</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B27">
-        <v>6</v>
-      </c>
-      <c r="C27" s="6" t="s">
+    </row>
+    <row r="28" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A28" s="5" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A28" s="5" t="s">
+      <c r="B28">
+        <v>100</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="B28">
-        <v>20</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -1725,7 +1683,7 @@
         <v>45</v>
       </c>
       <c r="B29">
-        <v>5</v>
+        <v>1.96</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>46</v>
@@ -1736,68 +1694,14 @@
         <v>47</v>
       </c>
       <c r="B30">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A31" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B31">
-        <v>100</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A32" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B32">
-        <v>1.96</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="29" x14ac:dyDescent="0.35">
-      <c r="A33" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B33">
-        <v>25</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="58" x14ac:dyDescent="0.35">
-      <c r="A34" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B34" t="s">
-        <v>132</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B35" t="s">
-        <v>133</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="35" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="43" ht="19.5" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
completing all descriptions in control files, first version of training dataset ready for translation
</commit_message>
<xml_diff>
--- a/1_msr_creator/control_file_msr_creator.xlsx
+++ b/1_msr_creator/control_file_msr_creator.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/26001 MSR tutorial/1_msr_creator/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/MSR code repo/1_msr_creator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="180" documentId="13_ncr:1_{66067BA5-85F1-4566-9789-B17D8F553E15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88E9B0C5-8EE9-4459-9953-E7C1737280E5}"/>
+  <xr:revisionPtr revIDLastSave="243" documentId="13_ncr:1_{66067BA5-85F1-4566-9789-B17D8F553E15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BAE33B1C-7DCA-4051-A380-7E8581D6E2D8}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="paths" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="147">
   <si>
     <t>parameters</t>
   </si>
@@ -217,9 +217,6 @@
     <t>file_name_regions</t>
   </si>
   <si>
-    <t>Region names</t>
-  </si>
-  <si>
     <t>file_name_region_boundaries</t>
   </si>
   <si>
@@ -298,9 +295,6 @@
     <t>file_name_buffer_distance</t>
   </si>
   <si>
-    <t>Regions and the corresponding road and grid buffer distance.</t>
-  </si>
-  <si>
     <t>file_name_ghi_map</t>
   </si>
   <si>
@@ -409,14 +403,74 @@
     <t>buffer_distance</t>
   </si>
   <si>
-    <t>(for very rare cases, in case grid distance to be calculated w.r.t. neighbouring grid)</t>
+    <t>File name with region names (.csv)</t>
+  </si>
+  <si>
+    <t>File name with corresponding road and grid buffer distance per region (.csv)</t>
+  </si>
+  <si>
+    <t>File name of image carrying population density</t>
+  </si>
+  <si>
+    <t>File name of image carrying urban areas (for naming purposes; not needed for filtering)</t>
+  </si>
+  <si>
+    <t>File name of image carrying land cover</t>
+  </si>
+  <si>
+    <t>File name of image carrying elevation</t>
+  </si>
+  <si>
+    <t>File name of image carrying climate zones</t>
+  </si>
+  <si>
+    <t>File name of image carrying protected areas</t>
+  </si>
+  <si>
+    <t>File name of image carrying water bodies</t>
+  </si>
+  <si>
+    <t>File name of shapefile carrying road network</t>
+  </si>
+  <si>
+    <t>File name of shapefile carrying substations</t>
+  </si>
+  <si>
+    <t>File name of shapefile carrying transmission and distribution grid</t>
+  </si>
+  <si>
+    <t>File name of shapefile carrying transmission grid</t>
+  </si>
+  <si>
+    <t>File name of shapefile carrying distribution grid</t>
+  </si>
+  <si>
+    <t>File name of shapefile carrying transmission grid from neighbouring countries (for very rare cases, in case grid distance to be calculated w.r.t. neighbouring grid)</t>
+  </si>
+  <si>
+    <t>File name of image carrying wind speeds</t>
+  </si>
+  <si>
+    <t>File name of image carrying global horizontal irradiation</t>
+  </si>
+  <si>
+    <t>File name of image carrying direct normal irradiation</t>
+  </si>
+  <si>
+    <t>File name matching climate classes with descriptions (.csv)</t>
+  </si>
+  <si>
+    <t>File name matching land cover categories with descriptions (.csv)</t>
+  </si>
+  <si>
+    <t>source</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -463,6 +517,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -500,7 +561,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -559,6 +620,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -591,10 +655,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table5" displayName="Table5" ref="A1:C3" totalsRowShown="0">
   <autoFilter ref="A1:C3" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
@@ -608,11 +668,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table1" displayName="Table1" ref="A1:C22" totalsRowShown="0">
-  <autoFilter ref="A1:C22" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table1" displayName="Table1" ref="A1:D22" totalsRowShown="0">
+  <autoFilter ref="A1:D22" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="parameter"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="value"/>
+    <tableColumn id="4" xr3:uid="{995DA6CD-33D0-403B-BA92-9CB13FECDD90}" name="source"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -952,24 +1013,24 @@
     </row>
     <row r="2" spans="1:3" s="7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="7" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="B3" s="17" t="s">
-        <v>103</v>
-      </c>
       <c r="C3" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -985,15 +1046,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="38.1796875" style="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.453125" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="69.7265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="63.90625" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="77.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>49</v>
       </c>
@@ -1001,234 +1063,293 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>63</v>
       </c>
       <c r="B2" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3" s="21"/>
+      <c r="D3" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="B3" s="21" t="s">
-        <v>121</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" s="21" t="s">
+      <c r="C6" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="21" t="s">
+      <c r="C7" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B7" s="21" t="s">
+      <c r="C8" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B8" s="21" t="s">
+      <c r="C9" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B9" s="21" t="s">
+      <c r="C10" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B12" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B10" s="21" t="s">
+      <c r="C12" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>120</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B12" s="21" t="s">
+      <c r="C13" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B14" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="D14" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="5" t="s">
+      <c r="C15" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B16"/>
+      <c r="C16"/>
+      <c r="D16" s="22" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="C17" s="20"/>
+      <c r="D17" s="5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B18" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B15" s="21" t="s">
+      <c r="C18" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="B16"/>
-      <c r="C16" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B17" s="20" t="s">
-        <v>127</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="B18" s="21" t="s">
+      <c r="C19" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B20"/>
+      <c r="C20"/>
+      <c r="D20" s="5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B21" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="C18" s="5" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B19" s="21" t="s">
+      <c r="C21" s="20"/>
+      <c r="D21" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B22" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B20"/>
-      <c r="C20" s="5"/>
-    </row>
-    <row r="21" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="B21" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="C21" s="5"/>
-    </row>
-    <row r="22" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="B22" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="C22" s="5"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="5" t="s">
+        <v>145</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1265,7 +1386,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1276,7 +1397,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1287,7 +1408,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1298,7 +1419,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1336,7 +1457,7 @@
     </row>
     <row r="9" spans="1:3" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B9" s="8">
         <v>1</v>
@@ -1347,7 +1468,7 @@
     </row>
     <row r="10" spans="1:3" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B10" s="8">
         <v>1</v>
@@ -1471,7 +1592,7 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>13</v>

</xml_diff>